<commit_message>
docs(custdev): add Р23 to Excel spreadsheet
</commit_message>
<xml_diff>
--- a/internal-docs/cust-dev-result.xlsx
+++ b/internal-docs/cust-dev-result.xlsx
@@ -654,7 +654,7 @@
           <t>Кого опрашиваем (ICP)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Работающие/учащиеся Android-пользователи, 18–45 лет, которые периодически задумываются «почему сегодня так тяжело» и уже отслеживают хотя бы что-то (сон, шаги, настроение) — но не получают объяснений из этих данных</t>
         </is>
@@ -709,15 +709,15 @@
       <c r="C7" s="20" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Расскажи как проходит обычный день — работаешь, учишься, что делаешь вечером?</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Профиль и базовая ситуация: ритм жизни определяет ценность прогноза</t>
         </is>
@@ -727,12 +727,12 @@
       <c r="A10" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Можешь вспомнить последний раз, когда что-то в себе отслеживал — сон, настроение, шаги, калории?</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Есть ли опыт self-tracking: насколько аудитория уже знакома с темой</t>
         </is>
@@ -949,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="12" min="1" max="1"/>
@@ -2115,106 +2115,158 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Р21</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>03.10.2026</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Текстовая переписка</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Студент колледжа, 18–22 лет</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>Принципиальный скептик — проверка второго типа не-аудитории (≠ Р14)</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>«Навязывание контакта с программой — идея для тех кому это надо, но таких людей маловато». «Я сам пойму»</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
         <is>
           <t>Принципиальная самодостаточность — идеологический отказ от внешней рефлексии (другой тип чем Р14)</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="12" t="inlineStr">
         <is>
           <t>Нет. Зафиксирован второй тип не-аудитории: проблема есть, но внешняя помощь отвергается</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25" s="12" t="inlineStr">
         <is>
           <t>Не инвестировать в убеждение скептиков. Граница ICP: нужна ощущаемая проблема + открытость</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Р22</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>04.10.2026</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>Живое интервью</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>Фрилансер (ИИ/машинное обучение), 40–45 лет</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="12" t="inlineStr">
         <is>
           <t>Высокая саморефлексия, 15 лет самонаблюдения — проверка гипотезы о барьере логирования</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>«Логирование занимает столько же времени, сколько само действие». «Если бы оно напоминало — я бы сделал»</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="12" t="inlineStr">
         <is>
           <t>Сильнейшая PMF-формулировка: логирование = барьер сам по себе. Пассивный сбор убирает его полностью</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="12" t="inlineStr">
         <is>
           <t>Да + лид на супругу (проблемы с засыпанием). Механику не понял без объяснения</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="12" t="inlineStr">
         <is>
           <t>Экран «вот что приложение делает пока ты спишь». Лид: бессонница как отдельная точка входа</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Р23</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Живое интервью</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Офисная работа, ~30 лет, хобби (вязание)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Активный трекер (цикл 10 лет, сон ментально, шаги) без системного инсайта — проверка гипотезы о новизне</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Нашла Screen Time с третьей попытки. Дала бы доступ к экрану и сну ("ничего конфиденциального"). Страх "ноишки": ИИ-агент может спереть данные. Если ничего не нужно интегрировать — поставит</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Инсайт должен быть новым — если подтверждает самодиагноз ("нет самодисциплины") — перестанет пользоваться. Новый барьер: ИИ-агент как отдельный вектор угрозы. Первый запрос на streak-геймификацию</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Условно. Основное условие: неочевидный инсайт + нулевое трение настройки</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Промпт должен давать новое, не отражать известное. Объяснять что ИИ видит паттерны, не сырые данные. Streak-механика — потенциальный инструмент удержания (roadmap)</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2316,7 @@
         </is>
       </c>
       <c r="B3" s="24">
-        <f>COUNTA(Интервью!E5:E26)</f>
+        <f>COUNTA(Интервью!E5:E27)</f>
         <v/>
       </c>
     </row>
@@ -2275,7 +2327,7 @@
         </is>
       </c>
       <c r="B4" s="24">
-        <f>COUNTIF(Интервью!C5:C26,"Живое интервью")</f>
+        <f>COUNTIF(Интервью!C5:C27,"Живое интервью")</f>
         <v/>
       </c>
     </row>
@@ -2286,7 +2338,7 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>COUNTIF(Интервью!C5:C26,"Текстовая переписка")</f>
+        <f>COUNTIF(Интервью!C5:C27,"Текстовая переписка")</f>
         <v/>
       </c>
     </row>
@@ -2297,7 +2349,7 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>COUNTIF(Интервью!D5:D26,"Да")</f>
+        <f>COUNTIF(Интервью!D5:D27,"Да")</f>
         <v/>
       </c>
     </row>
@@ -2318,17 +2370,17 @@
           <t>Люди регулярно переживают «необъяснимые» плохие дни и хотят понять причину</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Подтверждена</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Р1, Р2, Р4, Р9, Р22</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Утренний прогноз формулируется как ответ на вопрос «почему сегодня может быть сложнее»</t>
         </is>
@@ -2473,7 +2525,7 @@
       <c r="D16" s="19" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Главные выводы</t>
         </is>

</xml_diff>

<commit_message>
docs(custdev): add interview #24 — transparency demand, app-list privacy, trust inversion
Р24 (remote dev, ~25-30, St. Petersburg): requires explanation button ("why this
forecast"), treats app list as intimate data, trusts small devs more than large ones
(already compromised), notes morning bad-day notification can feel like "piling on".
Repeating asks: computer data integration, tiered info depth, day-over-day trends.
</commit_message>
<xml_diff>
--- a/internal-docs/cust-dev-result.xlsx
+++ b/internal-docs/cust-dev-result.xlsx
@@ -949,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="12" min="1" max="1"/>
@@ -2219,54 +2219,106 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Р23</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>05.10.2026</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Живое интервью</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Офисная работа, ~30 лет, хобби (вязание)</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Активный трекер (цикл 10 лет, сон ментально, шаги) без системного инсайта — проверка гипотезы о новизне</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>Нашла Screen Time с третьей попытки. Дала бы доступ к экрану и сну ("ничего конфиденциального"). Страх "ноишки": ИИ-агент может спереть данные. Если ничего не нужно интегрировать — поставит</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="12" t="inlineStr">
         <is>
           <t>Инсайт должен быть новым — если подтверждает самодиагноз ("нет самодисциплины") — перестанет пользоваться. Новый барьер: ИИ-агент как отдельный вектор угрозы. Первый запрос на streak-геймификацию</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>Условно. Основное условие: неочевидный инсайт + нулевое трение настройки</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="12" t="inlineStr">
         <is>
           <t>Промпт должен давать новое, не отражать известное. Объяснять что ИИ видит паттерны, не сырые данные. Streak-механика — потенциальный инструмент удержания (roadmap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Р24</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Живое интервью</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>Разработчик (удалённо, Петербург), 25–30 лет</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Технически грамотный, активно тренируется (3-4 раза/нед), замечает паттерны (TikTok-ловушка, курение-триггер). Не смотрит Screen Time — "страшно". Проверка гипотезы о прозрачности прогноза</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Список приложений — "довольно интимная информация". Крупным компаниям доверяет меньше (уже скомпрометированы), маленькому разработчику — больше. Хочет кнопку "почему такой прогноз" — видеть данные-основу. Попробовал бы</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Нестандартная логика доверия: большой = меньше доверия. Список приложений = интимная зона (первый кто явно назвал). Запрос на прозрачность прогноза. Уведомление "тяжёлый день" может "добивать" если уже плохо</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>Да, условно. Требует объяснения прогноза и нулевого навязывания. Экранное время перетекает между устройствами — блокировка одного не решает задачу</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>Кнопка "почему такой прогноз" — приоритет. Тон утренней нотификации: не "добивать". Дозированная информация (кратко/подробно). Тренды по дням. Объединение с данными компьютера — повторный запрос</t>
         </is>
       </c>
     </row>
@@ -2309,6 +2361,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="13">
       <c r="A3" s="18" t="inlineStr">
         <is>
@@ -2327,7 +2380,7 @@
         </is>
       </c>
       <c r="B4" s="24">
-        <f>COUNTIF(Интервью!C5:C27,"Живое интервью")</f>
+        <f>COUNTIF(Интервью!C5:C28,"Живое интервью")</f>
         <v/>
       </c>
     </row>
@@ -2338,7 +2391,7 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>COUNTIF(Интервью!C5:C27,"Текстовая переписка")</f>
+        <f>COUNTIF(Интервью!C5:C28,"Текстовая переписка")</f>
         <v/>
       </c>
     </row>
@@ -2349,7 +2402,7 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>COUNTIF(Интервью!D5:D27,"Да")</f>
+        <f>COUNTIF(Интервью!D5:D28,"Да")</f>
         <v/>
       </c>
     </row>
@@ -2364,6 +2417,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="13">
       <c r="A9" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(custdev): add interview #25 — zero-tracker user, built-in health competitor question
Р25 (female, work+side job): never used any health tracker, didn't know phone already
collects this data. Patterns already articulated without the app (introversion, cycle,
work stress). Key signal: must answer "why better than built-in Health?" in onboarding.
Curiosity hook: exact screen time in numbers. Deletes on ads.
</commit_message>
<xml_diff>
--- a/internal-docs/cust-dev-result.xlsx
+++ b/internal-docs/cust-dev-result.xlsx
@@ -949,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="12" min="1" max="1"/>
@@ -2319,6 +2319,58 @@
       <c r="J28" s="12" t="inlineStr">
         <is>
           <t>Кнопка "почему такой прогноз" — приоритет. Тон утренней нотификации: не "добивать". Дозированная информация (кратко/подробно). Тренды по дням. Объединение с данными компьютера — повторный запрос</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>Р25</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Текстовая переписка</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Женщина, возраст н/у, работа + подработка</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Нулевой пользователь трекеров — не знала о встроенных функциях здоровья. Паттерны осознаны самостоятельно (интроверсия, цикл, рабочий стресс). Проверка восприятия у нетехничной аудитории без контекста</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Не знала о существовании Screen Time. Паттерны и так очевидны. Любопытство: сколько конкретно времени занял телефон. Дала разрешение — первое приложение которому давала. Иногда игнорирует вечерний чекин</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Ключевой вопрос: чем лучше встроенной программы здоровья в телефоне? Паттерны уже артикулированы без продукта. «Ничего не смущает, но непонятно как поможет». Высокий барьер разрешений (давала впервые)</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>Условно. Нужно объяснить отличие от встроенного Health. Удалит при рекламе</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Onboarding должен отвечать на вопрос «чем лучше встроенного». Не пытаться открыть паттерны — они уже известны. Акцент на количественной стороне (сколько конкретно часов) как точке входа для нетрекеров</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2432,7 @@
         </is>
       </c>
       <c r="B4" s="24">
-        <f>COUNTIF(Интервью!C5:C28,"Живое интервью")</f>
+        <f>COUNTIF(Интервью!C5:C29,"Живое интервью")</f>
         <v/>
       </c>
     </row>
@@ -2391,7 +2443,7 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>COUNTIF(Интервью!C5:C28,"Текстовая переписка")</f>
+        <f>COUNTIF(Интервью!C5:C29,"Текстовая переписка")</f>
         <v/>
       </c>
     </row>
@@ -2402,7 +2454,7 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>COUNTIF(Интервью!D5:D28,"Да")</f>
+        <f>COUNTIF(Интервью!D5:D29,"Да")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(custdev): add interview #26 — passive-collection ideal ICP, AI training data barrier
Р26 (female, hybrid work, active lifestyle): multi-tracker (wearable + emotion diary +
cycle), loves causal analysis, refuses manual input — perfect passive-collection ICP.
Two strong product questions: (1) AI training on raw screen data feels invasive —
need explicit stat-only disclaimer; (2) aggregated screen time without context is
irrelevant (book browser ≠ TikTok browser). Potential referral.
</commit_message>
<xml_diff>
--- a/internal-docs/cust-dev-result.xlsx
+++ b/internal-docs/cust-dev-result.xlsx
@@ -949,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="12" min="1" max="1"/>
@@ -2371,6 +2371,58 @@
       <c r="J29" s="12" t="inlineStr">
         <is>
           <t>Onboarding должен отвечать на вопрос «чем лучше встроенного». Не пытаться открыть паттерны — они уже известны. Акцент на количественной стороне (сколько конкретно часов) как точке входа для нетрекеров</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Р26</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>06.10.2026</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Текстовая переписка</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Женщина, возраст н/у, гибридная работа, активный ЗОЖ (теннис, сноуборд, вело)</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Продвинутый мультитрекер: браслет (сон/пульс/восстановление) + дневник эмоций + цикл. Аналитический склад, встроенная привычка анализировать. Принципиально против ручного ввода — идеальный ICP</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>«Если данные не нужно вносить — интересно причинно-следственные связи». Screen Time смотрит осознанно. Барьер: обучение AI на сырых данных экрана (фото, переписки). Прогноз непонятен без механики. Умный вопрос: браузер с книгой ≠ браузер с видосиками — агрегат нерелевантен без контекста</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>Идеальная формулировка ценности пассивного сбора: «браслет сам считает, думает». Первый кто поставил вопрос о нерелевантности агрегированного экранного времени без контекста. Барьер: обучение AI моделей на сырых данных</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>Условно — потенциальный реферал. Нужна прозрачность: (1) только статистика, не скриншоты; (2) объяснение механики прогноза</t>
+        </is>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>Явный дисклеймер: сбор только статистический (время в приложениях), не скриншоты/переписки, не обучение модели. Объяснять механику прогноза на онбординге. Контекст использования важнее агрегата времени</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2484,7 @@
         </is>
       </c>
       <c r="B4" s="24">
-        <f>COUNTIF(Интервью!C5:C29,"Живое интервью")</f>
+        <f>COUNTIF(Интервью!C5:C30,"Живое интервью")</f>
         <v/>
       </c>
     </row>
@@ -2443,7 +2495,7 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>COUNTIF(Интервью!C5:C29,"Текстовая переписка")</f>
+        <f>COUNTIF(Интервью!C5:C30,"Текстовая переписка")</f>
         <v/>
       </c>
     </row>
@@ -2454,7 +2506,7 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>COUNTIF(Интервью!D5:D29,"Да")</f>
+        <f>COUNTIF(Интервью!D5:D30,"Да")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(custdev): add interview #27 — self-sufficient analyst, micromanagement as top stopper
Р27 (male, work+training+creativity): self-declared full tracker, already solves bad
days independently (decompress + sport). Utilitarian permissions barrier — will grant
if concrete benefit explained upfront. Key phrase: "extra micromanagement" as deletion
trigger — product must inform, not instruct. Borderline ICP: no felt need for external
insight.
</commit_message>
<xml_diff>
--- a/internal-docs/cust-dev-result.xlsx
+++ b/internal-docs/cust-dev-result.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ICP и вопросы" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Интервью" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итоги" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Инструкция" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ICP и вопросы" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Интервью" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Итоги" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -949,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="12" min="1" max="1"/>
@@ -2423,6 +2423,58 @@
       <c r="J30" s="12" t="inlineStr">
         <is>
           <t>Явный дисклеймер: сбор только статистический (время в приложениях), не скриншоты/переписки, не обучение модели. Объяснять механику прогноза на онбординге. Контекст использования важнее агрегата времени</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Р27</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>07.10.2026</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Текстовая переписка</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Мужчина, возраст н/у, работа + тренировки + творчество</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Самодекларированный трекер — «всегда отслеживаю всё». Следит за Screen Time. Паттерны уже осознаны и решены самостоятельно (разгрузка + спорт). Прагматичный аналитик</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>Утилитарный барьер разрешений: «дам если понадобится для конкретной задачи». «Возможно, если почувствую необходимость» — не чувствует сейчас. Главный стоп: «лишний микроменеджмент»</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>«Микроменеджмент» — ёмкая формулировка запрета: продукт должен информировать, не инструктировать. Пограничный ICP: инструменты уже есть. Утилитарный барьер — разрешение нужно обосновывать до запроса</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>Пограничный — нет ощущения необходимости. Реферал нет</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Продукт информирует, не управляет — формулировка для UX-принципа. Разрешение запрашивать с объяснением конкретной пользы ДО запроса. Не навязывать уведомления и действия</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2536,7 @@
         </is>
       </c>
       <c r="B4" s="24">
-        <f>COUNTIF(Интервью!C5:C30,"Живое интервью")</f>
+        <f>COUNTIF(Интервью!C5:C31,"Живое интервью")</f>
         <v/>
       </c>
     </row>
@@ -2495,7 +2547,7 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>COUNTIF(Интервью!C5:C30,"Текстовая переписка")</f>
+        <f>COUNTIF(Интервью!C5:C31,"Текстовая переписка")</f>
         <v/>
       </c>
     </row>
@@ -2506,7 +2558,7 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>COUNTIF(Интервью!D5:D30,"Да")</f>
+        <f>COUNTIF(Интервью!D5:D31,"Да")</f>
         <v/>
       </c>
     </row>

</xml_diff>